<commit_message>
12tak ki booking and last recent data
</commit_message>
<xml_diff>
--- a/Client Name & NTN List.xlsx
+++ b/Client Name & NTN List.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\786\Desktop\Elite Traders\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\786\Desktop\Elite-Git\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DB53610-3FB0-4DB7-8381-A0893D878641}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9F2C853-700D-47A2-8917-18E83836A4D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,12 +22,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -2522,14 +2516,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2537,17 +2531,13 @@
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2855,10 +2845,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
     </row>
     <row r="4" spans="2:6" ht="13" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
@@ -4313,7 +4303,7 @@
       </c>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:6" ht="13" x14ac:dyDescent="0.3">
       <c r="B95" s="2">
         <f t="shared" si="1"/>
         <v>91</v>
@@ -4484,7 +4474,7 @@
       <c r="D105" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="E105" s="11">
+      <c r="E105" s="9">
         <v>300426949714</v>
       </c>
       <c r="F105" s="3"/>
@@ -7481,7 +7471,7 @@
       </c>
       <c r="F292" s="3"/>
     </row>
-    <row r="293" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="293" spans="2:6" ht="13" x14ac:dyDescent="0.3">
       <c r="B293" s="2">
         <f t="shared" si="4"/>
         <v>289</v>
@@ -9321,7 +9311,7 @@
       </c>
       <c r="F407" s="3"/>
     </row>
-    <row r="408" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="408" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B408" s="2">
         <f t="shared" si="6"/>
         <v>404</v>
@@ -9337,7 +9327,7 @@
       </c>
       <c r="F408" s="3"/>
     </row>
-    <row r="409" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="409" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B409" s="2">
         <f t="shared" si="6"/>
         <v>405</v>
@@ -9353,7 +9343,7 @@
       </c>
       <c r="F409" s="3"/>
     </row>
-    <row r="410" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="410" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B410" s="2">
         <f t="shared" si="6"/>
         <v>406</v>
@@ -9369,7 +9359,7 @@
       </c>
       <c r="F410" s="3"/>
     </row>
-    <row r="411" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="411" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B411" s="2">
         <f t="shared" si="6"/>
         <v>407</v>
@@ -9385,7 +9375,7 @@
       </c>
       <c r="F411" s="3"/>
     </row>
-    <row r="412" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="412" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B412" s="2">
         <f t="shared" si="6"/>
         <v>408</v>
@@ -9401,7 +9391,7 @@
       </c>
       <c r="F412" s="3"/>
     </row>
-    <row r="413" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="413" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B413" s="2">
         <f t="shared" si="6"/>
         <v>409</v>
@@ -9417,7 +9407,7 @@
       </c>
       <c r="F413" s="3"/>
     </row>
-    <row r="414" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="414" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B414" s="2">
         <f t="shared" si="6"/>
         <v>410</v>
@@ -9433,7 +9423,7 @@
       </c>
       <c r="F414" s="3"/>
     </row>
-    <row r="415" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="415" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B415" s="2">
         <f t="shared" si="6"/>
         <v>411</v>
@@ -9449,7 +9439,7 @@
       </c>
       <c r="F415" s="3"/>
     </row>
-    <row r="416" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="416" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B416" s="2">
         <f t="shared" si="6"/>
         <v>412</v>
@@ -9465,7 +9455,7 @@
       </c>
       <c r="F416" s="3"/>
     </row>
-    <row r="417" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="417" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B417" s="2">
         <f t="shared" si="6"/>
         <v>413</v>
@@ -9481,7 +9471,7 @@
       </c>
       <c r="F417" s="3"/>
     </row>
-    <row r="418" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="418" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B418" s="2">
         <f t="shared" si="6"/>
         <v>414</v>
@@ -9497,7 +9487,7 @@
       </c>
       <c r="F418" s="3"/>
     </row>
-    <row r="419" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="419" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B419" s="2">
         <f t="shared" si="6"/>
         <v>415</v>
@@ -9513,7 +9503,7 @@
       </c>
       <c r="F419" s="3"/>
     </row>
-    <row r="420" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="420" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B420" s="2">
         <f t="shared" si="6"/>
         <v>416</v>
@@ -9529,7 +9519,7 @@
       </c>
       <c r="F420" s="3"/>
     </row>
-    <row r="421" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="421" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B421" s="2">
         <f t="shared" si="6"/>
         <v>417</v>
@@ -9545,7 +9535,7 @@
       </c>
       <c r="F421" s="3"/>
     </row>
-    <row r="422" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="422" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B422" s="2">
         <f t="shared" si="6"/>
         <v>418</v>
@@ -9561,7 +9551,7 @@
       </c>
       <c r="F422" s="3"/>
     </row>
-    <row r="423" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="423" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B423" s="2">
         <f t="shared" si="6"/>
         <v>419</v>
@@ -9577,7 +9567,7 @@
       </c>
       <c r="F423" s="3"/>
     </row>
-    <row r="424" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="424" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B424" s="2">
         <f t="shared" si="6"/>
         <v>420</v>
@@ -9593,7 +9583,7 @@
       </c>
       <c r="F424" s="3"/>
     </row>
-    <row r="425" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="425" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B425" s="2">
         <f t="shared" si="6"/>
         <v>421</v>
@@ -9609,7 +9599,7 @@
       </c>
       <c r="F425" s="3"/>
     </row>
-    <row r="426" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="426" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B426" s="2">
         <f t="shared" si="6"/>
         <v>422</v>
@@ -9625,7 +9615,7 @@
       </c>
       <c r="F426" s="3"/>
     </row>
-    <row r="427" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="427" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B427" s="2">
         <f t="shared" si="6"/>
         <v>423</v>
@@ -9641,7 +9631,7 @@
       </c>
       <c r="F427" s="3"/>
     </row>
-    <row r="428" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="428" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B428" s="2">
         <f t="shared" si="6"/>
         <v>424</v>
@@ -9657,7 +9647,7 @@
       </c>
       <c r="F428" s="3"/>
     </row>
-    <row r="429" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="429" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B429" s="2">
         <f t="shared" si="6"/>
         <v>425</v>
@@ -9673,7 +9663,7 @@
       </c>
       <c r="F429" s="3"/>
     </row>
-    <row r="430" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="430" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B430" s="2">
         <f t="shared" si="6"/>
         <v>426</v>
@@ -9689,7 +9679,7 @@
       </c>
       <c r="F430" s="3"/>
     </row>
-    <row r="431" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="431" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B431" s="2">
         <f t="shared" si="6"/>
         <v>427</v>
@@ -9705,7 +9695,7 @@
       </c>
       <c r="F431" s="3"/>
     </row>
-    <row r="432" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="432" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B432" s="2">
         <f t="shared" si="6"/>
         <v>428</v>
@@ -9721,7 +9711,7 @@
       </c>
       <c r="F432" s="3"/>
     </row>
-    <row r="433" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="433" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B433" s="2">
         <f t="shared" si="6"/>
         <v>429</v>
@@ -9737,7 +9727,7 @@
       </c>
       <c r="F433" s="3"/>
     </row>
-    <row r="434" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="434" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B434" s="2">
         <f t="shared" si="6"/>
         <v>430</v>
@@ -9753,7 +9743,7 @@
       </c>
       <c r="F434" s="3"/>
     </row>
-    <row r="435" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="435" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B435" s="2">
         <f t="shared" si="6"/>
         <v>431</v>
@@ -9769,7 +9759,7 @@
       </c>
       <c r="F435" s="3"/>
     </row>
-    <row r="436" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="436" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B436" s="2">
         <f t="shared" si="6"/>
         <v>432</v>
@@ -9785,7 +9775,7 @@
       </c>
       <c r="F436" s="3"/>
     </row>
-    <row r="437" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="437" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B437" s="2">
         <f t="shared" si="6"/>
         <v>433</v>
@@ -9801,7 +9791,7 @@
       </c>
       <c r="F437" s="3"/>
     </row>
-    <row r="438" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="438" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B438" s="2">
         <f t="shared" si="6"/>
         <v>434</v>
@@ -9817,7 +9807,7 @@
       </c>
       <c r="F438" s="3"/>
     </row>
-    <row r="439" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="439" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B439" s="2">
         <f t="shared" si="6"/>
         <v>435</v>
@@ -9833,7 +9823,7 @@
       </c>
       <c r="F439" s="3"/>
     </row>
-    <row r="440" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="440" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B440" s="2">
         <f t="shared" si="6"/>
         <v>436</v>
@@ -9849,7 +9839,7 @@
       </c>
       <c r="F440" s="3"/>
     </row>
-    <row r="441" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="441" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B441" s="2">
         <f t="shared" si="6"/>
         <v>437</v>
@@ -9865,7 +9855,7 @@
       </c>
       <c r="F441" s="3"/>
     </row>
-    <row r="442" spans="2:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="442" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B442" s="2">
         <f t="shared" si="6"/>
         <v>438</v>
@@ -11033,7 +11023,7 @@
       </c>
       <c r="F514" s="3"/>
     </row>
-    <row r="515" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="515" spans="2:6" ht="13" x14ac:dyDescent="0.3">
       <c r="B515" s="2">
         <f t="shared" si="7"/>
         <v>511</v>
@@ -11065,7 +11055,7 @@
       </c>
       <c r="F516" s="3"/>
     </row>
-    <row r="517" spans="2:6" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="517" spans="2:6" ht="13" x14ac:dyDescent="0.3">
       <c r="B517" s="2">
         <f t="shared" si="7"/>
         <v>513</v>
@@ -12381,10 +12371,10 @@
       <c r="B599" s="6">
         <v>595</v>
       </c>
-      <c r="C599" s="8" t="s">
+      <c r="C599" s="1" t="s">
         <v>794</v>
       </c>
-      <c r="D599" s="9" t="s">
+      <c r="D599" s="2" t="s">
         <v>795</v>
       </c>
       <c r="E599" s="5"/>
@@ -12393,7 +12383,7 @@
       <c r="B600" s="6">
         <v>596</v>
       </c>
-      <c r="C600" s="8" t="s">
+      <c r="C600" s="1" t="s">
         <v>796</v>
       </c>
       <c r="D600" s="6" t="s">
@@ -12411,7 +12401,7 @@
       <c r="C602" s="4" t="s">
         <v>800</v>
       </c>
-      <c r="D602" s="10" t="s">
+      <c r="D602" s="8" t="s">
         <v>799</v>
       </c>
     </row>
@@ -12419,13 +12409,13 @@
       <c r="B603">
         <v>334</v>
       </c>
-      <c r="C603" s="12" t="s">
+      <c r="C603" s="10" t="s">
         <v>802</v>
       </c>
       <c r="D603" t="s">
         <v>803</v>
       </c>
-      <c r="E603" s="13">
+      <c r="E603" s="11">
         <v>3277876171384</v>
       </c>
     </row>
@@ -12433,13 +12423,13 @@
       <c r="B604">
         <v>263</v>
       </c>
-      <c r="C604" s="12" t="s">
+      <c r="C604" s="10" t="s">
         <v>804</v>
       </c>
-      <c r="D604" s="14" t="s">
+      <c r="D604" s="12" t="s">
         <v>805</v>
       </c>
-      <c r="E604" s="13">
+      <c r="E604" s="11">
         <v>3520210170957</v>
       </c>
     </row>
@@ -12447,41 +12437,10 @@
   <autoFilter ref="B4:F604" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="1">
       <filters>
-        <filter val="JALAL SONS  (COLLEGE ROAD) 02"/>
-        <filter val="Jalal sons  (Izmair Town) 01"/>
-        <filter val="Jalal sons (Askari 10 F sector ) 01"/>
-        <filter val="JALAL SONS (ASKARI 11 B BLOCK) 02"/>
-        <filter val="JALAL SONS (AYUBIA) 02"/>
-        <filter val="JALAL SONS (Bahira Orchard) 01"/>
-        <filter val="Jalal Sons (Bahria Town)  01"/>
-        <filter val="JALAL SONS (C BLOCK MODEL TOWN) 02"/>
-        <filter val="JALAL SONS (DHA C BLOCK,PHASE 6) 02"/>
-        <filter val="JALAL SONS (DHA PH IV) 02"/>
-        <filter val="JALAL SONS (DHA PH V) 02"/>
-        <filter val="JALAL SONS (DHA Y BLOCK) 02"/>
-        <filter val="JALAL SONS (EME) 02"/>
-        <filter val="JALAL SONS (FAISAL TOWN) 02"/>
-        <filter val="Jalal Sons (H Block) 01"/>
-        <filter val="JALAL SONS (HUSSAIN CHOWK GULBERG III) 02"/>
-        <filter val="JALAL SONS (IQBAL TOWN) 02"/>
-        <filter val="Jalal Sons (J.T Shadewal) 01"/>
-        <filter val="JALAL SONS (JOHER TOWN) 02"/>
-        <filter val="Jalal Sons (Lake City) 01"/>
-        <filter val="Jalal sons (Main Market) 01"/>
-        <filter val="JALAL SONS (MODEL TOWN LINK ROAD) 02"/>
-        <filter val="Jalal Sons (PAF Market) 01 main Market"/>
-        <filter val="JALAL SONS (PARAGON CITY) 02"/>
-        <filter val="JALAL SONS (PH VI) 02"/>
-        <filter val="JALAL SONS (PHASE 8 EX PARK VIEW) 02"/>
-        <filter val="JALAL SONS (REVAZ GARDEN) 02"/>
-        <filter val="JALAL SONS (SHADMAN) 02"/>
-        <filter val="JALAL SONS (SHAUKAT KHANUM) 02"/>
-        <filter val="JALAL SONS (STATE LIFE) 02"/>
-        <filter val="JALAL SONS (TALWAR CHOWK) 02"/>
-        <filter val="JALAL SONS (VALENCIA TOWN) 02"/>
-        <filter val="JALAL SONS (WAPDA TOWN) 02"/>
-        <filter val="JALAL SONS (XX) 02"/>
-        <filter val="Jalal Sons Askari X (01)"/>
+        <filter val="AL KHAN BAKERS (NESPAK)"/>
+        <filter val="Gourmet (Pak Arab)"/>
+        <filter val="ORGANICS (PAK HEIGHTS BUILDING)"/>
+        <filter val="PAK MADINA SUPER STORE (BEGAM KOT)"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:F598">

</xml_diff>